<commit_message>
Assignment Day 30 : Listeners, Reporting, and Environment
</commit_message>
<xml_diff>
--- a/src/test/resources/data/products-data-test.xlsx
+++ b/src/test/resources/data/products-data-test.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>productName</t>
   </si>
@@ -39,9 +39,6 @@
   </si>
   <si>
     <t>single</t>
-  </si>
-  <si>
-    <t>sauce-labs-bike-light</t>
   </si>
   <si>
     <t>sauce-labs-bolt-t-shirt</t>
@@ -1206,8 +1203,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="5" outlineLevelCol="1"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="33.859375" customWidth="1"/>
   </cols>
@@ -1233,15 +1230,15 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1249,15 +1246,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>